<commit_message>
Corregir dimension de puerta desactualizada (100x200 a 80x210cm) en todos los documentos
</commit_message>
<xml_diff>
--- a/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
+++ b/02_Proveedores/Fichas_Proveedores_Pausa_Maule.xlsx
@@ -923,7 +923,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Puerta Pino Radiata Italia 100x200cm</t>
+          <t>Puerta Pino Radiata Italia 80x210cm</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>https://www.easy.cl/puerta-pino-radiata-italia-100x200-cm-moldupanel-1274901/p</t>
+          <t>https://www.easy.cl/puerta-pino-radiata-italia-80x210-cm-moldupanel-1246767/p</t>
         </is>
       </c>
     </row>

</xml_diff>